<commit_message>
Renner-zoekfunctie toevoegen en riders.json uit Teams.xlsx genereren
- data/riders.json komt nu uit de volledige startlijst die is toegevoegd
  aan Teams.xlsx, i.p.v. een extern opgehaalde lijst
- Nieuwe sectie op de vergelijkingspagina: zoek een renner op rugnummer
  en zie het totaal aantal verzamelde fantasy-punten, de etappe-voor-etappe
  opbouw daarvan, en welke teams deze renner hebben opgenomen
- scoring.js: computeRiderPoints() berekent team-onafhankelijke
  renner-puntentotalen

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Teams.xlsx
+++ b/Teams.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TaimenBoumansiunxi\Claude Code\TDF 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86DD9F45-D9E1-458F-A389-5923A451EF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E81D2490-4583-449A-B6D3-1939139FAAD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{85F8A388-6F13-4681-8DB6-6246B2371A70}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="262">
   <si>
     <t>Thomas Blajul</t>
   </si>
@@ -201,13 +201,637 @@
   </si>
   <si>
     <t>213 BITTNER Pavel</t>
+  </si>
+  <si>
+    <t>UAE Team Emirates XRG</t>
+  </si>
+  <si>
+    <t>Pogačar, Tadej</t>
+  </si>
+  <si>
+    <t>Del Toro, Isaac</t>
+  </si>
+  <si>
+    <t>Grossschartner, Felix</t>
+  </si>
+  <si>
+    <t>McNulty, Brandon</t>
+  </si>
+  <si>
+    <t>Politt, Nils</t>
+  </si>
+  <si>
+    <t>Vermeersch, Florian</t>
+  </si>
+  <si>
+    <t>Wellens, Tim</t>
+  </si>
+  <si>
+    <t>Yates, Adam</t>
+  </si>
+  <si>
+    <t>Team Visma - Lease a Bike</t>
+  </si>
+  <si>
+    <t>Vingegaard, Jonas</t>
+  </si>
+  <si>
+    <t>Affini, Edoardo</t>
+  </si>
+  <si>
+    <t>Armirail, Bruno</t>
+  </si>
+  <si>
+    <t>Campenaerts, Victor</t>
+  </si>
+  <si>
+    <t>Hagenes, Per Strand</t>
+  </si>
+  <si>
+    <t>Jorgenson, Matteo</t>
+  </si>
+  <si>
+    <t>Kuss, Sepp</t>
+  </si>
+  <si>
+    <t>Piganzoli, Davide</t>
+  </si>
+  <si>
+    <t>Red Bull - BORA - hansgrohe</t>
+  </si>
+  <si>
+    <t>Evenepoel, Remco</t>
+  </si>
+  <si>
+    <t>Cattaneo, Mattia</t>
+  </si>
+  <si>
+    <t>Denz, Nico</t>
+  </si>
+  <si>
+    <t>Hindley, Jai</t>
+  </si>
+  <si>
+    <t>Lipowitz, Florian</t>
+  </si>
+  <si>
+    <t>Tratnik, Jan</t>
+  </si>
+  <si>
+    <t>Dijke, Tim van</t>
+  </si>
+  <si>
+    <t>Gils, Maxim Van</t>
+  </si>
+  <si>
+    <t>Lidl - Trek</t>
+  </si>
+  <si>
+    <t>Ayuso, Juan</t>
+  </si>
+  <si>
+    <t>Gee-West, Derek</t>
+  </si>
+  <si>
+    <t>Pedersen, Mads</t>
+  </si>
+  <si>
+    <t>Simmons, Quinn</t>
+  </si>
+  <si>
+    <t>Skjelmose, Mattias</t>
+  </si>
+  <si>
+    <t>Skujiņš, Toms</t>
+  </si>
+  <si>
+    <t>Vacek, Mathias</t>
+  </si>
+  <si>
+    <t>Verona, Carlos</t>
+  </si>
+  <si>
+    <t>EF Education - EasyPost</t>
+  </si>
+  <si>
+    <t>Carapaz, Richard</t>
+  </si>
+  <si>
+    <t>Asgreen, Kasper</t>
+  </si>
+  <si>
+    <t>Baudin, Alex</t>
+  </si>
+  <si>
+    <t>Healy, Ben</t>
+  </si>
+  <si>
+    <t>Quinn, Sean</t>
+  </si>
+  <si>
+    <t>Steinhauser, Georg</t>
+  </si>
+  <si>
+    <t>Valgren, Michael</t>
+  </si>
+  <si>
+    <t>Walker, Max</t>
+  </si>
+  <si>
+    <t>Decathlon CMA CGM Team</t>
+  </si>
+  <si>
+    <t>Seixas, Paul</t>
+  </si>
+  <si>
+    <t>Benoot, Tiesj</t>
+  </si>
+  <si>
+    <t>Bol, Cees</t>
+  </si>
+  <si>
+    <t>Hoole, Daan</t>
+  </si>
+  <si>
+    <t>Kooij, Olav</t>
+  </si>
+  <si>
+    <t>Paret-Peintre, Aurélien</t>
+  </si>
+  <si>
+    <t>Prodhomme, Nicolas</t>
+  </si>
+  <si>
+    <t>Riccitello, Matthew</t>
+  </si>
+  <si>
+    <t>XDS Astana Team</t>
+  </si>
+  <si>
+    <t>Higuita, Sergio</t>
+  </si>
+  <si>
+    <t>Ballerini, Davide</t>
+  </si>
+  <si>
+    <t>Gate, Aaron</t>
+  </si>
+  <si>
+    <t>Kanter, Max</t>
+  </si>
+  <si>
+    <t>Tejada, Harold</t>
+  </si>
+  <si>
+    <t>Teunissen, Mike</t>
+  </si>
+  <si>
+    <t>Velasco, Simone</t>
+  </si>
+  <si>
+    <t>Vinokurov, Nicolas</t>
+  </si>
+  <si>
+    <t>Bahrain Victorious</t>
+  </si>
+  <si>
+    <t>Martinez, Lenny</t>
+  </si>
+  <si>
+    <t>Bauhaus, Phil</t>
+  </si>
+  <si>
+    <t>Caruso, Damiano</t>
+  </si>
+  <si>
+    <t>Gradek, Kamil</t>
+  </si>
+  <si>
+    <t>Mohorič, Matej</t>
+  </si>
+  <si>
+    <t>Stannard, Robert</t>
+  </si>
+  <si>
+    <t>Tiberi, Antonio</t>
+  </si>
+  <si>
+    <t>Mechelen, Vlad Van</t>
+  </si>
+  <si>
+    <t>Netcompany INEOS</t>
+  </si>
+  <si>
+    <t>Bernal, Egan</t>
+  </si>
+  <si>
+    <t>Arensman, Thymen</t>
+  </si>
+  <si>
+    <t>Foss, Tobias</t>
+  </si>
+  <si>
+    <t>Ganna, Filippo</t>
+  </si>
+  <si>
+    <t>Godon, Dorian</t>
+  </si>
+  <si>
+    <t>Kwiatkowski, Michal</t>
+  </si>
+  <si>
+    <t>Tarling, Josh</t>
+  </si>
+  <si>
+    <t>Vauquelin, Kévin</t>
+  </si>
+  <si>
+    <t>Soudal - Quick-Step</t>
+  </si>
+  <si>
+    <t>Merlier, Tim</t>
+  </si>
+  <si>
+    <t>Eenkhoorn, Pascal</t>
+  </si>
+  <si>
+    <t>Paret-Peintre, Valentin</t>
+  </si>
+  <si>
+    <t>Stuyven, Jasper</t>
+  </si>
+  <si>
+    <t>Baarle, Dylan van</t>
+  </si>
+  <si>
+    <t>Lerberghe, Bert Van</t>
+  </si>
+  <si>
+    <t>Wilder, Ilan Van</t>
+  </si>
+  <si>
+    <t>Vervaeke, Louis</t>
+  </si>
+  <si>
+    <t>Alpecin - Premier Tech</t>
+  </si>
+  <si>
+    <t>Poel, Mathieu van der</t>
+  </si>
+  <si>
+    <t>Debruyne, Ramses</t>
+  </si>
+  <si>
+    <t>Dillier, Silvan</t>
+  </si>
+  <si>
+    <t>Marsman, Tim</t>
+  </si>
+  <si>
+    <t>Philipsen, Jasper</t>
+  </si>
+  <si>
+    <t>Planckaert, Edward</t>
+  </si>
+  <si>
+    <t>Rickaert, Jonas</t>
+  </si>
+  <si>
+    <t>Verstrynge, Emiel</t>
+  </si>
+  <si>
+    <t>Team Jayco AlUla</t>
+  </si>
+  <si>
+    <t>O'Connor, Ben</t>
+  </si>
+  <si>
+    <t>Ackermann, Pascal</t>
+  </si>
+  <si>
+    <t>Durbridge, Luke</t>
+  </si>
+  <si>
+    <t>Engelhardt, Felix</t>
+  </si>
+  <si>
+    <t>Matthews, Michael</t>
+  </si>
+  <si>
+    <t>O'Brien, Kelland</t>
+  </si>
+  <si>
+    <t>Plapp, Luke</t>
+  </si>
+  <si>
+    <t>Schmid, Mauro</t>
+  </si>
+  <si>
+    <t>Uno-X Mobility</t>
+  </si>
+  <si>
+    <t>Johannessen, Tobias</t>
+  </si>
+  <si>
+    <t>Abrahamsen, Jonas</t>
+  </si>
+  <si>
+    <t>Charmig, Anthon</t>
+  </si>
+  <si>
+    <t>Cort, Magnus</t>
+  </si>
+  <si>
+    <t>Johannessen, Anders</t>
+  </si>
+  <si>
+    <t>Skaarseth, Anders</t>
+  </si>
+  <si>
+    <t>Træen, Torstein</t>
+  </si>
+  <si>
+    <t>Wærenskjold, Søren</t>
+  </si>
+  <si>
+    <t>NSN Cycling Team</t>
+  </si>
+  <si>
+    <t>Girmay, Biniam</t>
+  </si>
+  <si>
+    <t>Askey, Lewis</t>
+  </si>
+  <si>
+    <t>Bennett, George</t>
+  </si>
+  <si>
+    <t>Frigo, Marco</t>
+  </si>
+  <si>
+    <t>Louvel, Matîs</t>
+  </si>
+  <si>
+    <t>Neilands, Krists</t>
+  </si>
+  <si>
+    <t>Stewart, Jake</t>
+  </si>
+  <si>
+    <t>Asbroeck, Tom Van</t>
+  </si>
+  <si>
+    <t>Movistar Team</t>
+  </si>
+  <si>
+    <t>Uijtdebroeks, Cian</t>
+  </si>
+  <si>
+    <t>Castrillo, Pablo</t>
+  </si>
+  <si>
+    <t>Cepeda, Jefferson Alveiro</t>
+  </si>
+  <si>
+    <t>García, Raúl</t>
+  </si>
+  <si>
+    <t>Hessmann, Michel</t>
+  </si>
+  <si>
+    <t>Oliveira, Nelson</t>
+  </si>
+  <si>
+    <t>Romo, Javier</t>
+  </si>
+  <si>
+    <t>Rubio, Einer</t>
+  </si>
+  <si>
+    <t>Lotto - Intermarché</t>
+  </si>
+  <si>
+    <t>Lie, Arnaud De</t>
+  </si>
+  <si>
+    <t>Artz, Huub</t>
+  </si>
+  <si>
+    <t>Berckmoes, Jenno</t>
+  </si>
+  <si>
+    <t>Craps, Lars</t>
+  </si>
+  <si>
+    <t>Slock, Liam</t>
+  </si>
+  <si>
+    <t>Eetvelt, Lennert Van</t>
+  </si>
+  <si>
+    <t>Veistroffer, Baptiste</t>
+  </si>
+  <si>
+    <t>Zimmermann, Georg</t>
+  </si>
+  <si>
+    <t>Cofidis</t>
+  </si>
+  <si>
+    <t>Izagirre, Ion</t>
+  </si>
+  <si>
+    <t>Allegaert, Piet</t>
+  </si>
+  <si>
+    <t>Aranburu, Alex</t>
+  </si>
+  <si>
+    <t>Biermans, Jenthe</t>
+  </si>
+  <si>
+    <t>Fretin, Milan</t>
+  </si>
+  <si>
+    <t>Kirsch, Alex</t>
+  </si>
+  <si>
+    <t>Page, Hugo</t>
+  </si>
+  <si>
+    <t>Thomas, Benjamin</t>
+  </si>
+  <si>
+    <t>Pinarello - Q36.5 Pro Cycling Team</t>
+  </si>
+  <si>
+    <t>Pidcock, Tom</t>
+  </si>
+  <si>
+    <t>Azparren, Xabier Mikel</t>
+  </si>
+  <si>
+    <t>Harper, Chris</t>
+  </si>
+  <si>
+    <t>Hermans, Quinten</t>
+  </si>
+  <si>
+    <t>Howson, Damien</t>
+  </si>
+  <si>
+    <t>Meurisse, Xandro</t>
+  </si>
+  <si>
+    <t>Moer, Brent Van</t>
+  </si>
+  <si>
+    <t>Wright, Fred</t>
+  </si>
+  <si>
+    <t>Groupama - FDJ United</t>
+  </si>
+  <si>
+    <t>Grégoire, Romain</t>
+  </si>
+  <si>
+    <t>Berthet, Clément</t>
+  </si>
+  <si>
+    <t>Braz Afonso, Clément</t>
+  </si>
+  <si>
+    <t>Costiou, Ewen</t>
+  </si>
+  <si>
+    <t>Germani, Lorenzo</t>
+  </si>
+  <si>
+    <t>Martin-Guyonnet, Guillaume</t>
+  </si>
+  <si>
+    <t>Pacher, Quentin</t>
+  </si>
+  <si>
+    <t>Russo, Clément</t>
+  </si>
+  <si>
+    <t>Tudor Pro Cycling Team</t>
+  </si>
+  <si>
+    <t>Alaphilippe, Julian</t>
+  </si>
+  <si>
+    <t>Kleijn, Arvid de</t>
+  </si>
+  <si>
+    <t>Haller, Marco</t>
+  </si>
+  <si>
+    <t>Hirschi, Marc</t>
+  </si>
+  <si>
+    <t>Pluimers, Rick</t>
+  </si>
+  <si>
+    <t>Storer, Michael</t>
+  </si>
+  <si>
+    <t>Trentin, Matteo</t>
+  </si>
+  <si>
+    <t>Voisard, Yannis</t>
+  </si>
+  <si>
+    <t>TotalEnergies</t>
+  </si>
+  <si>
+    <t>Jegat, Jordan</t>
+  </si>
+  <si>
+    <t>Breuillard, Nicolas</t>
+  </si>
+  <si>
+    <t>Delbove, Joris</t>
+  </si>
+  <si>
+    <t>Delettre, Alexandre</t>
+  </si>
+  <si>
+    <t>Guernalec, Thibault</t>
+  </si>
+  <si>
+    <t>Le Berre, Mathis</t>
+  </si>
+  <si>
+    <t>Turgis, Anthony</t>
+  </si>
+  <si>
+    <t>Vercher, Mattéo</t>
+  </si>
+  <si>
+    <t>Team Picnic PostNL</t>
+  </si>
+  <si>
+    <t>Barguil, Warren</t>
+  </si>
+  <si>
+    <t>Biesterbos, Frits</t>
+  </si>
+  <si>
+    <t>Bittner, Pavel</t>
+  </si>
+  <si>
+    <t>Degenkolb, John</t>
+  </si>
+  <si>
+    <t>Dhondt, Robbe</t>
+  </si>
+  <si>
+    <t>Märkl, Niklas</t>
+  </si>
+  <si>
+    <t>Berg, Julius van den</t>
+  </si>
+  <si>
+    <t>Broek, Frank van den</t>
+  </si>
+  <si>
+    <t>Caja Rural - Seguros RGA</t>
+  </si>
+  <si>
+    <t>Gaviria, Fernando</t>
+  </si>
+  <si>
+    <t>Balderstone, Abel</t>
+  </si>
+  <si>
+    <t>Berwick, Sebastian</t>
+  </si>
+  <si>
+    <t>Molenaar, Alex</t>
+  </si>
+  <si>
+    <t>Nicolau, Joel</t>
+  </si>
+  <si>
+    <t>Oldani, Stefano</t>
+  </si>
+  <si>
+    <t>Otruba, Jakub</t>
+  </si>
+  <si>
+    <t>Parra, José Félix</t>
+  </si>
+  <si>
+    <t>OFFICIAL STARTLIST FULL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -223,13 +847,24 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Montserrat"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -245,9 +880,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -583,10 +1221,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA5C180D-B2B6-41F1-9140-280932E50656}">
-  <dimension ref="A4:I27"/>
+  <dimension ref="A4:I235"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="10" width="19" customWidth="1"/>
+    <col min="1" max="2" width="31.42578125" customWidth="1"/>
+    <col min="3" max="10" width="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -1201,6 +1840,1621 @@
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B27" s="1"/>
     </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="27" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B29" s="2"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
+        <v>1</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <v>2</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="27" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
+        <v>3</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>4</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
+        <v>5</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="2">
+        <v>6</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="2">
+        <v>7</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="2">
+        <v>8</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B38" s="2"/>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="2">
+        <v>11</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="2">
+        <v>12</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="2">
+        <v>13</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="2">
+        <v>14</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="2">
+        <v>15</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" s="2">
+        <v>16</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="2">
+        <v>17</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="2">
+        <v>18</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47" s="2"/>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="2">
+        <v>21</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="2">
+        <v>22</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" s="2">
+        <v>23</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="2">
+        <v>24</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" s="2">
+        <v>25</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" s="2">
+        <v>26</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" s="2">
+        <v>27</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" s="2">
+        <v>28</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B56" s="2"/>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" s="2">
+        <v>31</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" s="2">
+        <v>32</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="2">
+        <v>33</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="2">
+        <v>34</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="2">
+        <v>35</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="2">
+        <v>36</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" s="2">
+        <v>37</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" s="2">
+        <v>38</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A65" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B65" s="2"/>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" s="2">
+        <v>41</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" s="2">
+        <v>42</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" s="2">
+        <v>43</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="2">
+        <v>44</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="2">
+        <v>45</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" s="2">
+        <v>46</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="2">
+        <v>47</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="2">
+        <v>48</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A74" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B74" s="2"/>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" s="2">
+        <v>51</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" s="2">
+        <v>52</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" s="2">
+        <v>53</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" s="2">
+        <v>54</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79" s="2">
+        <v>55</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A80" s="2">
+        <v>56</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A81" s="2">
+        <v>57</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82" s="2">
+        <v>58</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B83" s="2"/>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84" s="2">
+        <v>61</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85" s="2">
+        <v>62</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" s="2">
+        <v>63</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87" s="2">
+        <v>64</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88" s="2">
+        <v>65</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89" s="2">
+        <v>66</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90" s="2">
+        <v>67</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91" s="2">
+        <v>68</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B92" s="2"/>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93" s="2">
+        <v>71</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94" s="2">
+        <v>72</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95" s="2">
+        <v>73</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A96" s="2">
+        <v>74</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97" s="2">
+        <v>75</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98" s="2">
+        <v>76</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A99" s="2">
+        <v>77</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A100" s="2">
+        <v>78</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A101" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B101" s="2"/>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A102" s="2">
+        <v>81</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103" s="2">
+        <v>82</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A104" s="2">
+        <v>83</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A105" s="2">
+        <v>84</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A106" s="2">
+        <v>85</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107" s="2">
+        <v>86</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A108" s="2">
+        <v>87</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109" s="2">
+        <v>88</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A110" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B110" s="2"/>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A111" s="2">
+        <v>91</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A112" s="2">
+        <v>92</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A113" s="2">
+        <v>93</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A114" s="2">
+        <v>94</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A115" s="2">
+        <v>95</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A116" s="2">
+        <v>96</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A117" s="2">
+        <v>97</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A118" s="2">
+        <v>98</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A119" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B119" s="2"/>
+    </row>
+    <row r="120" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A120" s="2">
+        <v>101</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A121" s="2">
+        <v>102</v>
+      </c>
+      <c r="B121" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A122" s="2">
+        <v>103</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A123" s="2">
+        <v>104</v>
+      </c>
+      <c r="B123" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A124" s="2">
+        <v>105</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A125" s="2">
+        <v>106</v>
+      </c>
+      <c r="B125" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A126" s="2">
+        <v>107</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A127" s="2">
+        <v>108</v>
+      </c>
+      <c r="B127" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A128" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B128" s="2"/>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A129" s="2">
+        <v>111</v>
+      </c>
+      <c r="B129" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A130" s="2">
+        <v>112</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A131" s="2">
+        <v>113</v>
+      </c>
+      <c r="B131" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A132" s="2">
+        <v>114</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A133" s="2">
+        <v>115</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A134" s="2">
+        <v>116</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A135" s="2">
+        <v>117</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A136" s="2">
+        <v>118</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A137" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B137" s="2"/>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A138" s="2">
+        <v>121</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A139" s="2">
+        <v>122</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A140" s="2">
+        <v>123</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A141" s="2">
+        <v>124</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A142" s="2">
+        <v>125</v>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A143" s="2">
+        <v>126</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A144" s="2">
+        <v>127</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A145" s="2">
+        <v>128</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A146" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="B146" s="2"/>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A147" s="2">
+        <v>131</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A148" s="2">
+        <v>132</v>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A149" s="2">
+        <v>133</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A150" s="2">
+        <v>134</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A151" s="2">
+        <v>135</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A152" s="2">
+        <v>136</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A153" s="2">
+        <v>137</v>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A154" s="2">
+        <v>138</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A155" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B155" s="2"/>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A156" s="2">
+        <v>141</v>
+      </c>
+      <c r="B156" s="2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A157" s="2">
+        <v>142</v>
+      </c>
+      <c r="B157" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A158" s="2">
+        <v>143</v>
+      </c>
+      <c r="B158" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A159" s="2">
+        <v>144</v>
+      </c>
+      <c r="B159" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A160" s="2">
+        <v>145</v>
+      </c>
+      <c r="B160" s="2" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A161" s="2">
+        <v>146</v>
+      </c>
+      <c r="B161" s="2" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A162" s="2">
+        <v>147</v>
+      </c>
+      <c r="B162" s="2" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A163" s="2">
+        <v>148</v>
+      </c>
+      <c r="B163" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A164" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="B164" s="2"/>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A165" s="2">
+        <v>151</v>
+      </c>
+      <c r="B165" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A166" s="2">
+        <v>152</v>
+      </c>
+      <c r="B166" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A167" s="2">
+        <v>153</v>
+      </c>
+      <c r="B167" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A168" s="2">
+        <v>154</v>
+      </c>
+      <c r="B168" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A169" s="2">
+        <v>155</v>
+      </c>
+      <c r="B169" s="2" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A170" s="2">
+        <v>156</v>
+      </c>
+      <c r="B170" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A171" s="2">
+        <v>157</v>
+      </c>
+      <c r="B171" s="2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A172" s="2">
+        <v>158</v>
+      </c>
+      <c r="B172" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A173" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B173" s="2"/>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A174" s="2">
+        <v>161</v>
+      </c>
+      <c r="B174" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A175" s="2">
+        <v>162</v>
+      </c>
+      <c r="B175" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A176" s="2">
+        <v>163</v>
+      </c>
+      <c r="B176" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A177" s="2">
+        <v>164</v>
+      </c>
+      <c r="B177" s="2" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A178" s="2">
+        <v>165</v>
+      </c>
+      <c r="B178" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A179" s="2">
+        <v>166</v>
+      </c>
+      <c r="B179" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A180" s="2">
+        <v>167</v>
+      </c>
+      <c r="B180" s="2" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A181" s="2">
+        <v>168</v>
+      </c>
+      <c r="B181" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A182" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B182" s="2"/>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A183" s="2">
+        <v>171</v>
+      </c>
+      <c r="B183" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A184" s="2">
+        <v>172</v>
+      </c>
+      <c r="B184" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A185" s="2">
+        <v>173</v>
+      </c>
+      <c r="B185" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A186" s="2">
+        <v>174</v>
+      </c>
+      <c r="B186" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A187" s="2">
+        <v>175</v>
+      </c>
+      <c r="B187" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A188" s="2">
+        <v>176</v>
+      </c>
+      <c r="B188" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A189" s="2">
+        <v>177</v>
+      </c>
+      <c r="B189" s="2" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A190" s="2">
+        <v>178</v>
+      </c>
+      <c r="B190" s="2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A191" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B191" s="2"/>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A192" s="2">
+        <v>181</v>
+      </c>
+      <c r="B192" s="2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A193" s="2">
+        <v>182</v>
+      </c>
+      <c r="B193" s="2" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A194" s="2">
+        <v>183</v>
+      </c>
+      <c r="B194" s="2" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A195" s="2">
+        <v>184</v>
+      </c>
+      <c r="B195" s="2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A196" s="2">
+        <v>185</v>
+      </c>
+      <c r="B196" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A197" s="2">
+        <v>186</v>
+      </c>
+      <c r="B197" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A198" s="2">
+        <v>187</v>
+      </c>
+      <c r="B198" s="2" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A199" s="2">
+        <v>188</v>
+      </c>
+      <c r="B199" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A200" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B200" s="2"/>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A201" s="2">
+        <v>191</v>
+      </c>
+      <c r="B201" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A202" s="2">
+        <v>192</v>
+      </c>
+      <c r="B202" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A203" s="2">
+        <v>193</v>
+      </c>
+      <c r="B203" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A204" s="2">
+        <v>194</v>
+      </c>
+      <c r="B204" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A205" s="2">
+        <v>195</v>
+      </c>
+      <c r="B205" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A206" s="2">
+        <v>196</v>
+      </c>
+      <c r="B206" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A207" s="2">
+        <v>197</v>
+      </c>
+      <c r="B207" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A208" s="2">
+        <v>198</v>
+      </c>
+      <c r="B208" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A209" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B209" s="2"/>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A210" s="2">
+        <v>201</v>
+      </c>
+      <c r="B210" s="2" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A211" s="2">
+        <v>202</v>
+      </c>
+      <c r="B211" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A212" s="2">
+        <v>203</v>
+      </c>
+      <c r="B212" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A213" s="2">
+        <v>204</v>
+      </c>
+      <c r="B213" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A214" s="2">
+        <v>205</v>
+      </c>
+      <c r="B214" s="2" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A215" s="2">
+        <v>206</v>
+      </c>
+      <c r="B215" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A216" s="2">
+        <v>207</v>
+      </c>
+      <c r="B216" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A217" s="2">
+        <v>208</v>
+      </c>
+      <c r="B217" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A218" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B218" s="2"/>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A219" s="2">
+        <v>211</v>
+      </c>
+      <c r="B219" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A220" s="2">
+        <v>212</v>
+      </c>
+      <c r="B220" s="2" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A221" s="2">
+        <v>213</v>
+      </c>
+      <c r="B221" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A222" s="2">
+        <v>214</v>
+      </c>
+      <c r="B222" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A223" s="2">
+        <v>215</v>
+      </c>
+      <c r="B223" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A224" s="2">
+        <v>216</v>
+      </c>
+      <c r="B224" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A225" s="2">
+        <v>217</v>
+      </c>
+      <c r="B225" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A226" s="2">
+        <v>218</v>
+      </c>
+      <c r="B226" s="2" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2" ht="27" x14ac:dyDescent="0.25">
+      <c r="A227" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B227" s="2"/>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A228" s="2">
+        <v>221</v>
+      </c>
+      <c r="B228" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A229" s="2">
+        <v>222</v>
+      </c>
+      <c r="B229" s="2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A230" s="2">
+        <v>223</v>
+      </c>
+      <c r="B230" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A231" s="2">
+        <v>224</v>
+      </c>
+      <c r="B231" s="2" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A232" s="2">
+        <v>225</v>
+      </c>
+      <c r="B232" s="2" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A233" s="2">
+        <v>226</v>
+      </c>
+      <c r="B233" s="2" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A234" s="2">
+        <v>227</v>
+      </c>
+      <c r="B234" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A235" s="2">
+        <v>228</v>
+      </c>
+      <c r="B235" s="2" t="s">
+        <v>260</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>